<commit_message>
Fix workflow and test pipeline changes
</commit_message>
<xml_diff>
--- a/content_log.xlsx
+++ b/content_log.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -533,6 +533,28 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-10-06 12:03:27</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Is Common Lisp The BEST Programming Language?! 🚀 #TechNews #Programming #Lisp</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Hold up, tech enthusiasts! A bold claim is shaking the internet: Common Lisp is now the best programming language. Really? Let's dive in! Yep, we're talking about Lisp, a language from the 1950s! But don't dismiss it. Recent discussions highlight its incredible power, especially for complex systems and AI research. What makes it 'best'? Common Lisp offers unparalleled metaprogramming capabilities. Imagine a language that can literally write and modify itself while it's running! Then there's its incredible stability and flexibility. Programs written decades ago often still compile and run perfectly, a rare feat in the fast-paced tech world. While it might seem niche, Lisp powers critical systems and is making a quiet comeback in AI, scientific computing, and advanced software development. So, is Common Lisp the *best*? Its unique strengths are undeniable, but it's not for everyone. What do YOU think? Let us know in the comments!</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>tech, programming, commonlisp, lisp, developers, coding, softwaredevelopment, shorts, techtalk, ai, news</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fix multi-scene and text overlay pipeline scripts
</commit_message>
<xml_diff>
--- a/content_log.xlsx
+++ b/content_log.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -582,66 +582,110 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-10-06 10:45:12</t>
+          <t>2026-10-07 21:35:54</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Francis Halzen Wins Nobel Physics 2026! 🏆 #NobelPrize #Physics #IceCube #TechNews</t>
+          <t>GitHub Down? గిట్ హబ్ లో సమస్యలు! 🤯 #GitHub #TechNewsTelugu #TeluguShorts</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Breaking News, science fans! The Nobel Prize in Physics 2026 goes to Professor Francis Halzen! He's the genius behind the IceCube Neutrino Observatory. Halzen's team detects high-energy cosmic neutrinos – 'ghost particles' from exploding stars and black holes! This revolutionary work gives us a new way to literally 'see' the universe's most extreme events. It's a monumental leap for astrophysics, unraveling cosmic origins. What does this Nobel mean for our future understanding of space? Tell us in the comments! Congrats, Professor Halzen!</t>
+          <t>హేయ్ టెక్ ప్రియులారా! ఇప్పుడే ఒక హాట్ న్యూస్ తో మీ ముందుకు వచ్చాను. మీరు గిట్ హబ్ వాడుతున్నారా? అయితే మీకు నిన్నటి నుంచి చిన్నపాటి షాక్ తగిలి ఉండొచ్చు. అవును, గిట్ హబ్ లో కొన్ని సమస్యలు తలెత్తాయి. గిట్ ఆపరేషన్స్, పుల్ రిక్వెస్ట్‌లు, గిట్ హబ్ యాక్షన్స్ వంటి ముఖ్యమైన ఫీచర్లు పనిచేయడం లేదని చాలా మంది డెవలపర్లు కంప్లైంట్ చేశారు. దీని వల్ల ప్రాజెక్ట్ డెవలప్‌మెంట్‌లో కాస్త బ్రేక్ వచ్చింది. కానీ వర్రీ అవ్వకండి! గిట్ హబ్ టీమ్ ఈ సమస్యను గుర్తించి, వేగంగా పరిష్కరించడానికి పని చేస్తుంది. త్వరలోనే అంతా నార్మల్ అవుతుందని ఆశిద్దాం. మరిన్ని టెక్ అప్‌డేట్స్ కోసం మన ఛానెల్‌ని సబ్‌స్క్రైబ్ చేసుకోండి! మీరేమైనా సమస్యలు ఎదుర్కొన్నారా? కామెంట్స్ లో చెప్పండి!</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>tech, news, shorts, nobelprize, physics, francishalzen, icecube, neutrino, astrophysics, science, space, cosmos, innovation, discovery, 2026</t>
+          <t>tech, telugu, ai, news, shorts, github, coding, developers, git</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-10-06 13:35:16</t>
+          <t>2026-10-07 22:52:51</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Mistral Large 4 Just Dropped! 🤯 AI Just Got SMARTER! #MistralAI #TechNews #AINews #Shorts</t>
+          <t>వీసా, మాస్టర్‌కార్డ్, బ్యాంకులపై దావా! 🚨 ఏంటి కథ? #TechNewsTelugu #VisaMastercard</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Tech world, buckle up! Mistral AI just made a massive move, unleashing 'Mistral Large 4' – their most advanced and powerful language model to date! This isn't just another update; it's a significant leap forward, designed to redefine what's possible with generative AI. Mistral Large 4 is engineered for peak performance, boasting impressive reasoning abilities and a deep understanding of complex tasks. It's stepping onto the global stage, ready to challenge even the biggest names in the LLM space. Imagine faster development, more accurate results, and groundbreaking AI applications across industries. This new model promises unparalleled efficiency and cutting-edge capabilities. It’s set to empower developers and transform how we interact with intelligent systems. The future of AI is evolving fast, and Mistral Large 4 is leading the charge. What incredible things do you think this new model will enable? Let us know in the comments! Stay ahead of the curve!</t>
+          <t>నమస్తే టెక్ ప్రియులారా! ఆర్థిక ప్రపంచంలో ఇప్పుడు పెద్ద అలజడి! వీసా, మాస్టర్‌కార్డ్, ఇంకా కొన్ని ప్రముఖ బ్యాంకులు భారీ లీగల్ చిక్కుల్లో పడ్డాయి. అవును, మీరు విన్నది నిజమే! క్రెడిట్ కార్డ్ లావాదేవీలపై వ్యాపారుల నుండి 'అన్యాయమైన' ఫీజులు వసూలు చేస్తున్నాయంటూ వాటిపై కొత్తగా దావా వేయబడింది. ఈ 'యాంటీకాంపిటీటివ్' ఫీజుల వల్ల వ్యాపారాలు కార్డు పేమెంట్స్ ప్రాసెస్ చేయడానికి భారీగా ఖర్చు చేయాల్సి వస్తుంది. చివరికి, ఈ భారం వినియోగదారులైన మనపైనే పడుతుందని నిపుణులు అంటున్నారు. మరి ఈ కేసు ఫలితం ఏమవుతుంది? బ్యాంకింగ్ రంగంలో ఎలాంటి మార్పులు వస్తాయో చూడాలి. ఈ విషయంపై మీ అభిప్రాయం ఏంటి? కామెంట్ల రూపంలో మాకు తెలియజేయండి! మన ఛానెల్‌ని సబ్స్క్రైబ్ చేసుకోవడం మర్చిపోకండి!</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>tech, ai, news, shorts, MistralAI, LLM, ArtificialIntelligence, ML, GenAI, Innovation</t>
+          <t>tech, telugu, news, shorts, visa, mastercard, banks, lawsuit, financialnews, techintelugu, business, consumerrights</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-10-07 15:32:10</t>
+          <t>2026-10-08 07:16:48</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>GitHub Glitch! 🚨 Devs, Did You Notice? #GitHubDown #TechNews #DevLife</t>
+          <t>సరికొత్త క్లాడ్ హైకు 5.5 AI | Anthropic కొత్త మోడల్ వచ్చేసింది! 🚀 #ClaudeHaiku #AI</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Hey devs, quick heads-up! GitHub just had a significant incident. If you faced issues with your Git operations, Pull Requests, or even GitHub Actions, you weren't alone. For a period, many developers experienced disruptions across these critical services. GitHub's status page confirmed the problem, affecting millions of projects globally. While they worked quickly to address it, it was a stark reminder of our reliance on these platforms. Always check GitHub's status page during outages! What's your backup plan when GitHub goes down? Let us know in the comments! Stay updated with the latest tech news right here.</t>
+          <t>హే టెక్ ప్రియులారా! AI ప్రపంచంలో మరో సంచలనానికి స్వాగతం! Anthropic నుండి సరికొత్త Claude Haiku 5.5 AI మోడల్ వచ్చేసింది. ఇది మునుపటి వెర్షన్ల కంటే చాలా వేగంగా, తక్కువ ఖర్చుతో పనిచేస్తుంది. మీ రోజువారీ AI పనులని మరింత సులభతరం చేస్తుంది. డెవలపర్స్, బిజినెస్ ల కోసం ఇది ఒక గేమ్ చేంజర్. క్లిష్టమైన డేటా అనాలిసిస్, కస్టమర్ సపోర్ట్, కోడింగ్ అసిస్టెన్స్ లాంటి వాటికి పర్ఫెక్ట్. రియల్ టైమ్ ప్రాసెసింగ్ సామర్థ్యంతో, Haiku 5.5 మీ ఉత్పాదకతను అమాంతం పెంచుతుంది. ఇది నిజంగా వేగం, సామర్థ్యం యొక్క అద్భుతమైన కలయిక. మీ ప్రాజెక్ట్స్ మరింత వేగంగా పూర్తవుతాయి. మరిన్ని టెక్ అప్డేట్స్ కోసం మా ఛానెల్ ని సబ్స్క్రైబ్ చేసుకోండి! Claude Haiku 5.5 గురించి మీరేమనుకుంటున్నారు? కామెంట్స్ లో చెప్పండి! తెలుగులో మరిన్ని టెక్ న్యూస్ కోసం చూస్తూ ఉండండి!</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>tech, news, github, developers, programming, coding, devops, shorts, outage, git, pullrequests, githubactions, incident</t>
+          <t>tech, telugu, ai, news, shorts, ClaudeHaiku, Anthropic, AIModel, TechNews, TeluguTech, ArtificialIntelligence, AIUpdate</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-10-08 07:33:09</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Claude Haiku 5.5: వేగవంతమైన, చవకైన AI వచ్చేసింది! 🚀 #AI #TeluguTech</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>హేయ్ టెక్ లవర్స్! AI ప్రపంచంలో మరో సంచలనం! Anthropic నుండి సరికొత్త Claude Haiku 5.5 వచ్చేసింది! గతంలో కంటే ఇంకా వేగంగా, చాలా తక్కువ ఖర్చుతో పనిచేసే ఈ AI మోడల్, చిన్న వ్యాపారాలకు, డెవలపర్‌లకు నిజంగా గేమ్-ఛేంజర్. కోడింగ్, కంటెంట్ క్రియేషన్, డేటా అనాలిసిస్.. ఇలా ఎన్నో పనులను క్షణాల్లో చేసేస్తుంది. ఇకపై AI శక్తి అందరికీ అందుబాటులోకి వస్తుంది. క్లాడ్ హైకు 5.5 సామర్థ్యాన్ని చూసి తీరాల్సిందే! మరిన్ని ఆసక్తికరమైన టెక్ అప్‌డేట్‌ల కోసం వెంటనే మన ఛానెల్‌ని సబ్‌స్క్రైబ్ చేసుకోండి!</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>tech, telugu, ai, news, shorts, claude haiku, anthropic, artificial intelligence, ai models, telugu tech news, fast ai, cost effective ai</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-10-08 07:42:54</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Claude Haiku 5.5: కొత్త AI వచ్చేసింది! 🚀🔥 | Anthropic AI Update #TeluguTech</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>ఒక అదిరిపోయే AI అప్డేట్! Anthropic నుండి సరికొత్త Claude Haiku 5.5 వచ్చేసింది! మీరు నమ్మలేరు... ఇది మునుపటి కంటే రెండు రెట్లు వేగంగా పనిచేస్తుంది! అవును, రెండంతలు ఫాస్ట్! అంతేకాదు, ఇది మరింత స్మార్ట్, తక్కువ ధరలో ఎక్కువ పని చేస్తుంది. కోడింగ్, లాజిక్, డిఫరెంట్ భాషల్లో కూడా అద్భుతమైన పర్ఫార్మెన్స్! ఇది మీ AI ప్రాజెక్టులకు బెస్ట్ ఆప్షన్ కావచ్చు. మరింత సమాచారం కోసం Anthropic వెబ్సైట్ చూడండి! AI ప్రపంచంలో ఇది ఒక గేమ్ ఛేంజర్! మిస్ అవ్వకండి!</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>tech, telugu, ai, news, shorts, claudehaiku, anthropic, aitools, telugutech, latestai</t>
         </is>
       </c>
     </row>

</xml_diff>